<commit_message>
feat: actualización de proyecto sin seed.js
</commit_message>
<xml_diff>
--- a/Formatos/INVENTARIO 2024..xlsx
+++ b/Formatos/INVENTARIO 2024..xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rubi DGMC\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\OneDrive\Documents\ULA\ula_inventario\Formatos\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBA510F2-B0E4-4E10-9C4C-432986AA6380}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21600" windowHeight="9630" activeTab="1"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -19,6 +20,9 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -494,8 +498,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="8" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -543,6 +547,14 @@
       <sz val="8"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -799,10 +811,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="11"/>
@@ -1014,6 +1027,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1029,33 +1048,32 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{B9FCF885-6DE0-416D-AA5A-8524044630AC}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1075,19 +1093,25 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>371475</xdr:colOff>
+      <xdr:colOff>685800</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>314325</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>116012</xdr:rowOff>
+      <xdr:rowOff>144587</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
@@ -1107,7 +1131,7 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="504825" y="19050"/>
+          <a:off x="819150" y="47625"/>
           <a:ext cx="1152525" cy="1287587"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1155,7 +1179,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 1"/>
+        <xdr:cNvPr id="5" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
@@ -1228,7 +1258,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
@@ -1296,7 +1332,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 1"/>
+        <xdr:cNvPr id="3" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000003000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
@@ -1364,7 +1406,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 1"/>
+        <xdr:cNvPr id="4" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
@@ -1432,7 +1480,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 1"/>
+        <xdr:cNvPr id="5" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000005000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
@@ -1750,7 +1804,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:M63"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1845,34 +1899,34 @@
       <c r="L9" s="3"/>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B10" s="98" t="s">
+      <c r="B10" s="91" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="99"/>
-      <c r="D10" s="99"/>
-      <c r="E10" s="91" t="s">
+      <c r="C10" s="92"/>
+      <c r="D10" s="92"/>
+      <c r="E10" s="93" t="s">
         <v>3</v>
       </c>
-      <c r="F10" s="99" t="s">
+      <c r="F10" s="92" t="s">
         <v>4</v>
       </c>
-      <c r="G10" s="99" t="s">
+      <c r="G10" s="92" t="s">
         <v>5</v>
       </c>
-      <c r="H10" s="99" t="s">
+      <c r="H10" s="92" t="s">
         <v>6</v>
       </c>
-      <c r="I10" s="91" t="s">
+      <c r="I10" s="93" t="s">
         <v>7</v>
       </c>
-      <c r="J10" s="91" t="s">
+      <c r="J10" s="93" t="s">
         <v>8</v>
       </c>
-      <c r="K10" s="93" t="s">
+      <c r="K10" s="95" t="s">
         <v>9</v>
       </c>
-      <c r="L10" s="94"/>
-      <c r="M10" s="95"/>
+      <c r="L10" s="96"/>
+      <c r="M10" s="97"/>
     </row>
     <row r="11" spans="2:13" ht="36" x14ac:dyDescent="0.25">
       <c r="B11" s="4" t="s">
@@ -1884,19 +1938,19 @@
       <c r="D11" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E11" s="92"/>
+      <c r="E11" s="94"/>
       <c r="F11" s="100"/>
       <c r="G11" s="100"/>
       <c r="H11" s="100"/>
-      <c r="I11" s="92"/>
-      <c r="J11" s="92"/>
+      <c r="I11" s="94"/>
+      <c r="J11" s="94"/>
       <c r="K11" s="5" t="s">
         <v>13</v>
       </c>
       <c r="L11" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="M11" s="6" t="s">
+      <c r="M11" s="105" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1925,7 +1979,9 @@
       <c r="I12" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="J12" s="7"/>
+      <c r="J12" s="7">
+        <v>12345</v>
+      </c>
       <c r="K12" s="12" t="s">
         <v>26</v>
       </c>
@@ -1955,7 +2011,9 @@
       <c r="I13" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="J13" s="7"/>
+      <c r="J13" s="7">
+        <v>12345</v>
+      </c>
       <c r="K13" s="12" t="s">
         <v>26</v>
       </c>
@@ -2009,7 +2067,9 @@
       <c r="I15" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="J15" s="7"/>
+      <c r="J15" s="7">
+        <v>12345</v>
+      </c>
       <c r="K15" s="12" t="s">
         <v>26</v>
       </c>
@@ -2031,7 +2091,9 @@
       <c r="I16" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="J16" s="7"/>
+      <c r="J16" s="7">
+        <v>12345</v>
+      </c>
       <c r="K16" s="12" t="s">
         <v>26</v>
       </c>
@@ -2062,7 +2124,7 @@
       <c r="L17" s="10"/>
       <c r="M17" s="11"/>
     </row>
-    <row r="18" spans="2:13" ht="45" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:13" ht="30" x14ac:dyDescent="0.25">
       <c r="B18" s="19"/>
       <c r="C18" s="20"/>
       <c r="D18" s="20"/>
@@ -2079,7 +2141,7 @@
       <c r="I18" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="J18" s="7"/>
+      <c r="J18" s="104"/>
       <c r="K18" s="12" t="s">
         <v>26</v>
       </c>
@@ -2306,8 +2368,8 @@
         <v>61</v>
       </c>
       <c r="H27" s="31"/>
-      <c r="I27" s="96"/>
-      <c r="J27" s="97"/>
+      <c r="I27" s="101"/>
+      <c r="J27" s="102"/>
       <c r="K27" s="31"/>
       <c r="L27" s="31"/>
       <c r="M27" s="31"/>
@@ -2412,34 +2474,34 @@
       <c r="L42" s="3"/>
     </row>
     <row r="43" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B43" s="98" t="s">
+      <c r="B43" s="91" t="s">
         <v>2</v>
       </c>
-      <c r="C43" s="99"/>
-      <c r="D43" s="99"/>
-      <c r="E43" s="91" t="s">
+      <c r="C43" s="92"/>
+      <c r="D43" s="92"/>
+      <c r="E43" s="93" t="s">
         <v>3</v>
       </c>
-      <c r="F43" s="99" t="s">
+      <c r="F43" s="92" t="s">
         <v>4</v>
       </c>
-      <c r="G43" s="99" t="s">
+      <c r="G43" s="92" t="s">
         <v>5</v>
       </c>
-      <c r="H43" s="99" t="s">
+      <c r="H43" s="92" t="s">
         <v>6</v>
       </c>
-      <c r="I43" s="91" t="s">
+      <c r="I43" s="93" t="s">
         <v>7</v>
       </c>
-      <c r="J43" s="91" t="s">
+      <c r="J43" s="93" t="s">
         <v>8</v>
       </c>
-      <c r="K43" s="93" t="s">
+      <c r="K43" s="95" t="s">
         <v>9</v>
       </c>
-      <c r="L43" s="94"/>
-      <c r="M43" s="95"/>
+      <c r="L43" s="96"/>
+      <c r="M43" s="97"/>
     </row>
     <row r="44" spans="2:13" ht="36" x14ac:dyDescent="0.25">
       <c r="B44" s="4" t="s">
@@ -2451,12 +2513,12 @@
       <c r="D44" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E44" s="92"/>
+      <c r="E44" s="94"/>
       <c r="F44" s="100"/>
       <c r="G44" s="100"/>
       <c r="H44" s="100"/>
-      <c r="I44" s="92"/>
-      <c r="J44" s="92"/>
+      <c r="I44" s="94"/>
+      <c r="J44" s="94"/>
       <c r="K44" s="5" t="s">
         <v>13</v>
       </c>
@@ -2685,8 +2747,8 @@
       <c r="F60" s="34"/>
       <c r="G60" s="34"/>
       <c r="H60" s="34"/>
-      <c r="I60" s="101"/>
-      <c r="J60" s="102"/>
+      <c r="I60" s="98"/>
+      <c r="J60" s="99"/>
       <c r="K60" s="34"/>
       <c r="L60" s="34"/>
       <c r="M60" s="34"/>
@@ -2708,11 +2770,20 @@
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="D35:L35"/>
-    <mergeCell ref="D36:L36"/>
-    <mergeCell ref="F39:M39"/>
-    <mergeCell ref="B40:K40"/>
-    <mergeCell ref="B41:L41"/>
+    <mergeCell ref="D2:L2"/>
+    <mergeCell ref="D3:L3"/>
+    <mergeCell ref="F6:M6"/>
+    <mergeCell ref="B7:K7"/>
+    <mergeCell ref="B8:L8"/>
+    <mergeCell ref="I10:I11"/>
+    <mergeCell ref="J10:J11"/>
+    <mergeCell ref="K10:M10"/>
+    <mergeCell ref="I27:J27"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="F10:F11"/>
+    <mergeCell ref="G10:G11"/>
+    <mergeCell ref="H10:H11"/>
     <mergeCell ref="B43:D43"/>
     <mergeCell ref="E43:E44"/>
     <mergeCell ref="K43:M43"/>
@@ -2722,20 +2793,11 @@
     <mergeCell ref="H43:H44"/>
     <mergeCell ref="I43:I44"/>
     <mergeCell ref="J43:J44"/>
-    <mergeCell ref="I10:I11"/>
-    <mergeCell ref="J10:J11"/>
-    <mergeCell ref="K10:M10"/>
-    <mergeCell ref="I27:J27"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="F10:F11"/>
-    <mergeCell ref="G10:G11"/>
-    <mergeCell ref="H10:H11"/>
-    <mergeCell ref="D2:L2"/>
-    <mergeCell ref="D3:L3"/>
-    <mergeCell ref="F6:M6"/>
-    <mergeCell ref="B7:K7"/>
-    <mergeCell ref="B8:L8"/>
+    <mergeCell ref="D35:L35"/>
+    <mergeCell ref="D36:L36"/>
+    <mergeCell ref="F39:M39"/>
+    <mergeCell ref="B40:K40"/>
+    <mergeCell ref="B41:L41"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="85" orientation="landscape" verticalDpi="0" r:id="rId1"/>
@@ -2744,7 +2806,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B1:M126"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2840,34 +2902,34 @@
       <c r="L9" s="3"/>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B10" s="98" t="s">
+      <c r="B10" s="91" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="99"/>
-      <c r="D10" s="99"/>
-      <c r="E10" s="91" t="s">
+      <c r="C10" s="92"/>
+      <c r="D10" s="92"/>
+      <c r="E10" s="93" t="s">
         <v>3</v>
       </c>
-      <c r="F10" s="99" t="s">
+      <c r="F10" s="92" t="s">
         <v>4</v>
       </c>
-      <c r="G10" s="99" t="s">
+      <c r="G10" s="92" t="s">
         <v>5</v>
       </c>
-      <c r="H10" s="99" t="s">
+      <c r="H10" s="92" t="s">
         <v>6</v>
       </c>
-      <c r="I10" s="91" t="s">
+      <c r="I10" s="93" t="s">
         <v>7</v>
       </c>
-      <c r="J10" s="91" t="s">
+      <c r="J10" s="93" t="s">
         <v>8</v>
       </c>
-      <c r="K10" s="93" t="s">
+      <c r="K10" s="95" t="s">
         <v>9</v>
       </c>
-      <c r="L10" s="94"/>
-      <c r="M10" s="95"/>
+      <c r="L10" s="96"/>
+      <c r="M10" s="97"/>
     </row>
     <row r="11" spans="2:13" ht="23.25" x14ac:dyDescent="0.25">
       <c r="B11" s="4" t="s">
@@ -2879,12 +2941,12 @@
       <c r="D11" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E11" s="92"/>
+      <c r="E11" s="94"/>
       <c r="F11" s="100"/>
       <c r="G11" s="100"/>
       <c r="H11" s="100"/>
-      <c r="I11" s="92"/>
-      <c r="J11" s="92"/>
+      <c r="I11" s="94"/>
+      <c r="J11" s="94"/>
       <c r="K11" s="5" t="s">
         <v>13</v>
       </c>
@@ -3334,34 +3396,34 @@
       <c r="L38" s="3"/>
     </row>
     <row r="39" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B39" s="98" t="s">
+      <c r="B39" s="91" t="s">
         <v>2</v>
       </c>
-      <c r="C39" s="99"/>
-      <c r="D39" s="99"/>
-      <c r="E39" s="91" t="s">
+      <c r="C39" s="92"/>
+      <c r="D39" s="92"/>
+      <c r="E39" s="93" t="s">
         <v>3</v>
       </c>
-      <c r="F39" s="99" t="s">
+      <c r="F39" s="92" t="s">
         <v>4</v>
       </c>
-      <c r="G39" s="99" t="s">
+      <c r="G39" s="92" t="s">
         <v>5</v>
       </c>
-      <c r="H39" s="99" t="s">
+      <c r="H39" s="92" t="s">
         <v>6</v>
       </c>
-      <c r="I39" s="91" t="s">
+      <c r="I39" s="93" t="s">
         <v>7</v>
       </c>
-      <c r="J39" s="91" t="s">
+      <c r="J39" s="93" t="s">
         <v>8</v>
       </c>
-      <c r="K39" s="93" t="s">
+      <c r="K39" s="95" t="s">
         <v>9</v>
       </c>
-      <c r="L39" s="94"/>
-      <c r="M39" s="95"/>
+      <c r="L39" s="96"/>
+      <c r="M39" s="97"/>
     </row>
     <row r="40" spans="2:13" ht="23.25" x14ac:dyDescent="0.25">
       <c r="B40" s="4" t="s">
@@ -3373,12 +3435,12 @@
       <c r="D40" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E40" s="92"/>
+      <c r="E40" s="94"/>
       <c r="F40" s="100"/>
       <c r="G40" s="100"/>
       <c r="H40" s="100"/>
-      <c r="I40" s="92"/>
-      <c r="J40" s="92"/>
+      <c r="I40" s="94"/>
+      <c r="J40" s="94"/>
       <c r="K40" s="5" t="s">
         <v>13</v>
       </c>
@@ -3951,34 +4013,34 @@
       <c r="L76" s="3"/>
     </row>
     <row r="77" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B77" s="98" t="s">
+      <c r="B77" s="91" t="s">
         <v>2</v>
       </c>
-      <c r="C77" s="99"/>
-      <c r="D77" s="99"/>
-      <c r="E77" s="91" t="s">
+      <c r="C77" s="92"/>
+      <c r="D77" s="92"/>
+      <c r="E77" s="93" t="s">
         <v>3</v>
       </c>
-      <c r="F77" s="99" t="s">
+      <c r="F77" s="92" t="s">
         <v>4</v>
       </c>
-      <c r="G77" s="99" t="s">
+      <c r="G77" s="92" t="s">
         <v>5</v>
       </c>
-      <c r="H77" s="99" t="s">
+      <c r="H77" s="92" t="s">
         <v>6</v>
       </c>
-      <c r="I77" s="91" t="s">
+      <c r="I77" s="93" t="s">
         <v>7</v>
       </c>
-      <c r="J77" s="91" t="s">
+      <c r="J77" s="93" t="s">
         <v>8</v>
       </c>
-      <c r="K77" s="93" t="s">
+      <c r="K77" s="95" t="s">
         <v>9</v>
       </c>
-      <c r="L77" s="94"/>
-      <c r="M77" s="95"/>
+      <c r="L77" s="96"/>
+      <c r="M77" s="97"/>
     </row>
     <row r="78" spans="2:13" ht="36" x14ac:dyDescent="0.25">
       <c r="B78" s="4" t="s">
@@ -3990,12 +4052,12 @@
       <c r="D78" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E78" s="92"/>
+      <c r="E78" s="94"/>
       <c r="F78" s="100"/>
       <c r="G78" s="100"/>
       <c r="H78" s="100"/>
-      <c r="I78" s="92"/>
-      <c r="J78" s="92"/>
+      <c r="I78" s="94"/>
+      <c r="J78" s="94"/>
       <c r="K78" s="5" t="s">
         <v>13</v>
       </c>
@@ -4376,8 +4438,8 @@
       <c r="F94" s="34"/>
       <c r="G94" s="34"/>
       <c r="H94" s="34"/>
-      <c r="I94" s="101"/>
-      <c r="J94" s="102"/>
+      <c r="I94" s="98"/>
+      <c r="J94" s="99"/>
       <c r="K94" s="34"/>
       <c r="L94" s="34"/>
       <c r="M94" s="34"/>
@@ -4522,34 +4584,34 @@
       <c r="L111" s="3"/>
     </row>
     <row r="112" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B112" s="98" t="s">
+      <c r="B112" s="91" t="s">
         <v>2</v>
       </c>
-      <c r="C112" s="99"/>
-      <c r="D112" s="99"/>
-      <c r="E112" s="91" t="s">
+      <c r="C112" s="92"/>
+      <c r="D112" s="92"/>
+      <c r="E112" s="93" t="s">
         <v>3</v>
       </c>
-      <c r="F112" s="99" t="s">
+      <c r="F112" s="92" t="s">
         <v>4</v>
       </c>
-      <c r="G112" s="99" t="s">
+      <c r="G112" s="92" t="s">
         <v>5</v>
       </c>
-      <c r="H112" s="99" t="s">
+      <c r="H112" s="92" t="s">
         <v>6</v>
       </c>
-      <c r="I112" s="91" t="s">
+      <c r="I112" s="93" t="s">
         <v>7</v>
       </c>
-      <c r="J112" s="91" t="s">
+      <c r="J112" s="93" t="s">
         <v>8</v>
       </c>
-      <c r="K112" s="93" t="s">
+      <c r="K112" s="95" t="s">
         <v>9</v>
       </c>
-      <c r="L112" s="94"/>
-      <c r="M112" s="95"/>
+      <c r="L112" s="96"/>
+      <c r="M112" s="97"/>
     </row>
     <row r="113" spans="2:13" ht="36" x14ac:dyDescent="0.25">
       <c r="B113" s="4" t="s">
@@ -4561,12 +4623,12 @@
       <c r="D113" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E113" s="92"/>
+      <c r="E113" s="94"/>
       <c r="F113" s="100"/>
       <c r="G113" s="100"/>
       <c r="H113" s="100"/>
-      <c r="I113" s="92"/>
-      <c r="J113" s="92"/>
+      <c r="I113" s="94"/>
+      <c r="J113" s="94"/>
       <c r="K113" s="5" t="s">
         <v>13</v>
       </c>
@@ -4834,47 +4896,6 @@
     </row>
   </sheetData>
   <mergeCells count="53">
-    <mergeCell ref="B36:K36"/>
-    <mergeCell ref="B37:L37"/>
-    <mergeCell ref="B39:D39"/>
-    <mergeCell ref="E39:E40"/>
-    <mergeCell ref="F39:F40"/>
-    <mergeCell ref="G39:G40"/>
-    <mergeCell ref="H39:H40"/>
-    <mergeCell ref="I39:I40"/>
-    <mergeCell ref="J39:J40"/>
-    <mergeCell ref="K39:M39"/>
-    <mergeCell ref="D31:L31"/>
-    <mergeCell ref="D32:L32"/>
-    <mergeCell ref="F35:M35"/>
-    <mergeCell ref="I10:I11"/>
-    <mergeCell ref="J10:J11"/>
-    <mergeCell ref="K10:M10"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="F10:F11"/>
-    <mergeCell ref="G10:G11"/>
-    <mergeCell ref="H10:H11"/>
-    <mergeCell ref="D2:L2"/>
-    <mergeCell ref="D3:L3"/>
-    <mergeCell ref="F6:M6"/>
-    <mergeCell ref="B7:K7"/>
-    <mergeCell ref="B8:L8"/>
-    <mergeCell ref="D69:L69"/>
-    <mergeCell ref="D70:L70"/>
-    <mergeCell ref="F73:M73"/>
-    <mergeCell ref="B74:K74"/>
-    <mergeCell ref="B75:L75"/>
-    <mergeCell ref="I77:I78"/>
-    <mergeCell ref="J77:J78"/>
-    <mergeCell ref="K77:M77"/>
-    <mergeCell ref="I94:J94"/>
-    <mergeCell ref="D104:L104"/>
-    <mergeCell ref="B77:D77"/>
-    <mergeCell ref="E77:E78"/>
-    <mergeCell ref="F77:F78"/>
-    <mergeCell ref="G77:G78"/>
-    <mergeCell ref="H77:H78"/>
     <mergeCell ref="D105:L105"/>
     <mergeCell ref="F108:M108"/>
     <mergeCell ref="B109:K109"/>
@@ -4887,6 +4908,47 @@
     <mergeCell ref="I112:I113"/>
     <mergeCell ref="J112:J113"/>
     <mergeCell ref="K112:M112"/>
+    <mergeCell ref="I77:I78"/>
+    <mergeCell ref="J77:J78"/>
+    <mergeCell ref="K77:M77"/>
+    <mergeCell ref="I94:J94"/>
+    <mergeCell ref="D104:L104"/>
+    <mergeCell ref="B77:D77"/>
+    <mergeCell ref="E77:E78"/>
+    <mergeCell ref="F77:F78"/>
+    <mergeCell ref="G77:G78"/>
+    <mergeCell ref="H77:H78"/>
+    <mergeCell ref="D69:L69"/>
+    <mergeCell ref="D70:L70"/>
+    <mergeCell ref="F73:M73"/>
+    <mergeCell ref="B74:K74"/>
+    <mergeCell ref="B75:L75"/>
+    <mergeCell ref="D2:L2"/>
+    <mergeCell ref="D3:L3"/>
+    <mergeCell ref="F6:M6"/>
+    <mergeCell ref="B7:K7"/>
+    <mergeCell ref="B8:L8"/>
+    <mergeCell ref="D31:L31"/>
+    <mergeCell ref="D32:L32"/>
+    <mergeCell ref="F35:M35"/>
+    <mergeCell ref="I10:I11"/>
+    <mergeCell ref="J10:J11"/>
+    <mergeCell ref="K10:M10"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="F10:F11"/>
+    <mergeCell ref="G10:G11"/>
+    <mergeCell ref="H10:H11"/>
+    <mergeCell ref="B36:K36"/>
+    <mergeCell ref="B37:L37"/>
+    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="E39:E40"/>
+    <mergeCell ref="F39:F40"/>
+    <mergeCell ref="G39:G40"/>
+    <mergeCell ref="H39:H40"/>
+    <mergeCell ref="I39:I40"/>
+    <mergeCell ref="J39:J40"/>
+    <mergeCell ref="K39:M39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="80" orientation="landscape" r:id="rId1"/>

</xml_diff>